<commit_message>
Update date calculator to competition dates
</commit_message>
<xml_diff>
--- a/Utils/AutoDateCalculator.xlsx
+++ b/Utils/AutoDateCalculator.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="28623"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="29231"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Ahmad\F1tenth\icra2025_race\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Ahmad\F1tenth\icra2026_race\Utils\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9CDAE932-235D-4DBA-BFB2-F04DA3382A8C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4FFF6235-AA07-479E-B7D8-C513453F4E72}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="2240" yWindow="2240" windowWidth="25800" windowHeight="10010" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-105" yWindow="0" windowWidth="26010" windowHeight="21705" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -588,16 +588,16 @@
     <outlinePr summaryBelow="0"/>
   </sheetPr>
   <dimension ref="B1:D10"/>
-  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="13.81640625" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="20.1796875" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="28.6328125" style="1" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="13.54296875" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="13.85546875" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="21.42578125" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="32.7109375" style="1" customWidth="1"/>
+    <col min="4" max="4" width="13.5703125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="2:4" ht="18.75" customHeight="1" x14ac:dyDescent="0.35"/>
-    <row r="2" spans="2:4" ht="18.75" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="1" spans="2:4" ht="18.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="2" spans="2:4" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B2" s="2" t="s">
         <v>0</v>
       </c>
@@ -605,78 +605,78 @@
         <v>1</v>
       </c>
     </row>
-    <row r="3" spans="2:4" ht="18.75" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="3" spans="2:4" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B3" s="4" t="s">
         <v>2</v>
       </c>
       <c r="C3" s="8">
-        <v>45799</v>
+        <v>46177</v>
       </c>
       <c r="D3" s="5" t="s">
         <v>10</v>
       </c>
     </row>
-    <row r="4" spans="2:4" ht="18.75" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="4" spans="2:4" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B4" s="6" t="s">
         <v>3</v>
       </c>
       <c r="C4" s="9">
         <f>C3-1</f>
-        <v>45798</v>
-      </c>
-    </row>
-    <row r="5" spans="2:4" ht="18.75" customHeight="1" x14ac:dyDescent="0.35">
+        <v>46176</v>
+      </c>
+    </row>
+    <row r="5" spans="2:4" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B5" s="4" t="s">
         <v>4</v>
       </c>
       <c r="C5" s="8">
         <f>C4-1</f>
-        <v>45797</v>
-      </c>
-    </row>
-    <row r="6" spans="2:4" ht="18.75" customHeight="1" x14ac:dyDescent="0.35">
+        <v>46175</v>
+      </c>
+    </row>
+    <row r="6" spans="2:4" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B6" s="6" t="s">
         <v>5</v>
       </c>
       <c r="C6" s="9">
         <f>C5-1</f>
-        <v>45796</v>
-      </c>
-    </row>
-    <row r="7" spans="2:4" ht="18.75" customHeight="1" x14ac:dyDescent="0.35">
+        <v>46174</v>
+      </c>
+    </row>
+    <row r="7" spans="2:4" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B7" s="4" t="s">
         <v>6</v>
       </c>
       <c r="C7" s="8">
         <f>C6-35</f>
-        <v>45761</v>
-      </c>
-    </row>
-    <row r="8" spans="2:4" ht="18.75" customHeight="1" x14ac:dyDescent="0.35">
+        <v>46139</v>
+      </c>
+    </row>
+    <row r="8" spans="2:4" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B8" s="6" t="s">
         <v>7</v>
       </c>
       <c r="C8" s="9">
         <f>C7-2</f>
-        <v>45759</v>
-      </c>
-    </row>
-    <row r="9" spans="2:4" ht="18.75" customHeight="1" x14ac:dyDescent="0.35">
+        <v>46137</v>
+      </c>
+    </row>
+    <row r="9" spans="2:4" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B9" s="4" t="s">
         <v>8</v>
       </c>
       <c r="C9" s="8">
         <f>C8-26</f>
-        <v>45733</v>
-      </c>
-    </row>
-    <row r="10" spans="2:4" ht="18.75" customHeight="1" x14ac:dyDescent="0.35">
+        <v>46111</v>
+      </c>
+    </row>
+    <row r="10" spans="2:4" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B10" s="7" t="s">
         <v>9</v>
       </c>
       <c r="C10" s="10">
         <f>C9-47</f>
-        <v>45686</v>
+        <v>46064</v>
       </c>
     </row>
   </sheetData>

</xml_diff>